<commit_message>
Enhance BingX and MEXC crawler resilience, fix symbol mapping and update margin tiers data
</commit_message>
<xml_diff>
--- a/data/bingx_position_tier.xlsx
+++ b/data/bingx_position_tier.xlsx
@@ -10,6 +10,12 @@
     <sheet name="BTCUSDT" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="ETHUSDT" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="SOLUSDT" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="HYPEUSDT" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="DOGEUSDT" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="XRPUSDT" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ADAUSDT" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="SOXLUSDT" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MSTRUSDT" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1380,7 +1386,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>62x</t>
+          <t>50x</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1417,7 +1423,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>62x</t>
+          <t>50x</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1454,7 +1460,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>41x</t>
+          <t>50x</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1491,7 +1497,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>25x</t>
+          <t>50x</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1528,7 +1534,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>25x</t>
+          <t>50x</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1861,7 +1867,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>25x</t>
+          <t>20x</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1898,7 +1904,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>25x</t>
+          <t>20x</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1935,7 +1941,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>25x</t>
+          <t>20x</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1972,7 +1978,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>25x</t>
+          <t>20x</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2009,7 +2015,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>5x</t>
+          <t>7x</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2108,7 +2114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2203,7 +2209,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>13,000,000</t>
+          <t>17,000,000</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -2240,7 +2246,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>15,000,000</t>
+          <t>30,000,000</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2250,12 +2256,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>227,676</t>
+          <t>637,676</t>
         </is>
       </c>
     </row>
@@ -2277,22 +2283,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>30,000,000</t>
+          <t>60,000,000</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>15x</t>
+          <t>10x</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>527,676</t>
+          <t>1,837,676</t>
         </is>
       </c>
     </row>
@@ -2314,22 +2320,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>60,000,000</t>
+          <t>80,000,000</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>10x</t>
+          <t>5x</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>1,727,676</t>
+          <t>3,037,676</t>
         </is>
       </c>
     </row>
@@ -2351,22 +2357,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>80,000,000</t>
+          <t>100,000,000</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5x</t>
+          <t>4x</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>13.33%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2,927,676</t>
+          <t>5,701,676</t>
         </is>
       </c>
     </row>
@@ -2388,22 +2394,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>100,000,000</t>
+          <t>150,000,000</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4x</t>
+          <t>2x</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>13.33%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5,591,676</t>
+          <t>12,371,676</t>
         </is>
       </c>
     </row>
@@ -2425,7 +2431,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>150,000,000</t>
+          <t>300,000,000</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -2435,12 +2441,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>12,261,676</t>
+          <t>42,371,676</t>
         </is>
       </c>
     </row>
@@ -2462,22 +2468,790 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>300,000,000</t>
+          <t>400,000,000</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>1x</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>72,371,676</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>交易所</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>檔位</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>單位</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>倉位分級</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>最大槓桿</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>維持保證金率</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>維持金額(USDT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>檔位 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2,600,000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>100x</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.5000%</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>檔位 2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>5,000,000</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>14x</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>117,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>檔位 3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>27,730,000</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>10x</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>7.14%</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>224,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>檔位 4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>55,300,000</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>2x</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>8.33%</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>553,987</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>檔位 5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>58,040,000</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2x</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1,477,497</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>檔位 6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>59,540,000</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2x</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>12.50%</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2,928,497</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>檔位 7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>112,260,000</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2x</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>16.67%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>5,411,315</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>檔位 8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>116,760,000</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2x</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>14,762,573</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>檔位 9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>117,440,000</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2x</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>42,261,676</t>
+          <t>43,952,573</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>交易所</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>檔位</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>單位</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>倉位分級</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>最大槓桿</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>維持保證金率</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>維持金額(USDT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>檔位 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>190,000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>300x</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.1700%</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>檔位 2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>4,200,000</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>200x</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.2500%</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>檔位 3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>20,000,000</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>10x</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>199,652</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>檔位 4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>21,000,000</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>5x</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>11.50%</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1,499,652</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>檔位 5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>23,000,000</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>5x</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1,604,652</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>檔位 6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>25,000,000</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>5x</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>12.50%</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1,719,652</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>檔位 7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>27,000,000</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>5x</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>13%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1,844,652</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>檔位 8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>29,000,000</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>5x</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>13.50%</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1,979,652</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>檔位 9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>50,000,000</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>5x</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>3,864,652</t>
         </is>
       </c>
     </row>
@@ -2499,22 +3273,1447 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>400,000,000</t>
+          <t>100,000,000</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>2x</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>6,364,652</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>檔位 11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>200,000,000</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>1x</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>50%</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>72,261,676</t>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>31,364,652</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>交易所</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>檔位</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>單位</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>倉位分級</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>最大槓桿</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>維持保證金率</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>維持金額(USDT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>檔位 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>180,000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>300x</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.1700%</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>檔位 2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3,400,000</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>300x</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.2500%</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>檔位 3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>15,000,000</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>25x</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>59,644</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>檔位 4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>45,000,000</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>15x</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>7.14%</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>830,644</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>檔位 5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>60,000,000</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>6x</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2,117,644</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>檔位 6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>80,000,000</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>4x</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>12.50%</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>3,617,644</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>檔位 7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>100,000,000</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>3x</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>16.67%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>6,953,644</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>檔位 8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>250,000,000</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2x</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>15,283,644</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>檔位 9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>300,000,000</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1x</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>77,783,644</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>交易所</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>檔位</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>單位</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>倉位分級</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>最大槓桿</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>維持保證金率</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>維持金額(USDT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>檔位 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>84,000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>300x</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.1700%</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>檔位 2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3,500,000</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>300x</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.2500%</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>67.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>檔位 3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>15,000,000</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>10x</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>166,317.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>檔位 4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>20,000,000</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>5x</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>13.30%</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1,411,317.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>檔位 5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>30,000,000</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>4x</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2,751,317.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>檔位 6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>50,000,000</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2x</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>8,751,317.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>檔位 7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>100,000,000</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1x</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>13,751,317.2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>交易所</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>檔位</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>單位</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>倉位分級</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>最大槓桿</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>維持保證金率</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>維持金額(USDT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>檔位 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>47,000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>200x</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.2500%</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>檔位 2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>200,000</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>50x</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1.25%</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>470</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>檔位 3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1,000,000</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>25x</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2.50%</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2,970</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>檔位 4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>6,500,000</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>20x</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>27,970</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>檔位 5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>25,000,000</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>5x</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>16.67%</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>786,520</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>檔位 6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>50,000,000</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>4x</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2,869,020</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>檔位 7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>200,000,000</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2x</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>15,369,020</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>交易所</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>檔位</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>單位</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>倉位分級</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>最大槓桿</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>維持保證金率</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>維持金額(USDT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>檔位 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>51,000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>100x</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.5000%</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>檔位 2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>92,000</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>100x</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>檔位 3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>500,000</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>25x</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>3.33%</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2,398.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>檔位 4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2,000,000</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>15x</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>10,748.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>檔位 5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>5,000,000</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>10x</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>110,748.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>檔位 6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>10,000,000</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>5x</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>12.50%</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>235,748.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>檔位 7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>25,000,000</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>4x</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>16.67%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>652,748.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>檔位 8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>50,000,000</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2x</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2,735,248.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BingX</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>檔位 9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>100,000,000</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1x</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>15,235,248.6</t>
         </is>
       </c>
     </row>

</xml_diff>